<commit_message>
Fix TBD states: Ozurigbo Ugonna (Imo), Onowakpo Thomas (Delta), durable API backfill
- export_data.py: refactor party fallback into _match_api_member(); add
  backfill_member_api() that fills missing/TBD state (house) and state +
  district (senate, from senatorial_zone) using the same PLAC members API
- Source fixes: senate csv Onowakpo row had party 'APC' misaligned into
  Official Name with TBD state/district -> proper name, Delta, Delta South;
  house excel Ozurigbo Ugonna State TBD -> Imo
- Remove unused root-level duplicate source files; repoint dev scripts to
  data/ versions
- house.json/senate.json regenerated: 0 TBD states remain
</commit_message>
<xml_diff>
--- a/data/house_of_reps_master_final.xlsx
+++ b/data/house_of_reps_master_final.xlsx
@@ -477,7 +477,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>/data/legislator_images/1.jpg?v=7</t>
@@ -508,7 +507,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>/data/legislator_images/2.jpg?v=7</t>
@@ -539,7 +537,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>/data/legislator_images/3.jpg?v=7</t>
@@ -570,7 +567,6 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>/data/legislator_images/4.jpg?v=7</t>
@@ -601,7 +597,6 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>/data/legislator_images/5.jpg?v=7</t>
@@ -632,7 +627,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>/data/legislator_images/6.jpg?v=7</t>
@@ -663,7 +657,6 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>/data/legislator_images/7.jpg?v=7</t>
@@ -694,7 +687,6 @@
           <t>Federal Capital Territory</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>/data/legislator_images/8.jpg?v=7</t>
@@ -725,7 +717,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>/data/legislator_images/9.jpg?v=7</t>
@@ -756,7 +747,6 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>/data/legislator_images/10.jpg?v=7</t>
@@ -787,7 +777,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>/data/legislator_images/11.jpg?v=7</t>
@@ -818,7 +807,6 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>/data/legislator_images/12.jpg?v=7</t>
@@ -849,7 +837,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>/data/legislator_images/13.jpg?v=7</t>
@@ -880,7 +867,6 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>/data/legislator_images/14.jpg?v=7</t>
@@ -911,7 +897,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>/data/legislator_images/15.jpg?v=7</t>
@@ -942,7 +927,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>/data/legislator_images/16.jpg?v=7</t>
@@ -973,7 +957,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>/data/legislator_images/17.jpg?v=7</t>
@@ -1004,7 +987,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>/data/legislator_images/18.jpg?v=7</t>
@@ -1035,7 +1017,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>/data/legislator_images/19.jpg?v=7</t>
@@ -1066,7 +1047,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>/data/legislator_images/20.jpg?v=7</t>
@@ -1097,7 +1077,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>/data/legislator_images/21.jpg?v=7</t>
@@ -1128,7 +1107,6 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>/data/legislator_images/22.jpg?v=7</t>
@@ -1159,7 +1137,6 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>/data/legislator_images/23.jpg?v=7</t>
@@ -1190,7 +1167,6 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>/data/legislator_images/24.jpg?v=7</t>
@@ -1221,7 +1197,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>/data/legislator_images/25.jpg?v=7</t>
@@ -1252,7 +1227,6 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>/data/legislator_images/26.jpg?v=7</t>
@@ -1318,7 +1292,6 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>/data/legislator_images/28.jpg?v=7</t>
@@ -1349,7 +1322,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>/data/legislator_images/29.jpg?v=7</t>
@@ -1380,7 +1352,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>/data/legislator_images/30.jpg?v=7</t>
@@ -1411,7 +1382,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>/data/legislator_images/31.jpg?v=7</t>
@@ -1442,7 +1412,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>/data/legislator_images/32.jpg?v=7</t>
@@ -1508,7 +1477,6 @@
           <t>Bayelsa</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>/data/legislator_images/34.jpg?v=7</t>
@@ -1539,7 +1507,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>/data/legislator_images/35.jpg?v=7</t>
@@ -1570,7 +1537,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>/data/legislator_images/36.jpg?v=7</t>
@@ -1601,7 +1567,6 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>/data/legislator_images/37.jpg?v=7</t>
@@ -1632,7 +1597,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>/data/legislator_images/38.jpg?v=7</t>
@@ -1663,7 +1627,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
           <t>/data/legislator_images/39.jpg?v=7</t>
@@ -1694,7 +1657,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>/data/legislator_images/40.jpg?v=7</t>
@@ -1725,7 +1687,6 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>/data/legislator_images/41.jpg?v=7</t>
@@ -1756,7 +1717,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>/data/legislator_images/42.jpg?v=7</t>
@@ -1787,7 +1747,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>/data/legislator_images/43.jpg?v=7</t>
@@ -1818,7 +1777,6 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>/data/legislator_images/44.jpg?v=7</t>
@@ -1849,7 +1807,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>/data/legislator_images/45.jpg?v=7</t>
@@ -1880,7 +1837,6 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>/data/legislator_images/46.jpg?v=7</t>
@@ -1911,7 +1867,6 @@
           <t>Cross River</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>/data/legislator_images/47.jpg?v=7</t>
@@ -1942,7 +1897,6 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>/data/legislator_images/48.jpg?v=7</t>
@@ -1973,7 +1927,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>/data/legislator_images/49.jpg?v=7</t>
@@ -2004,7 +1957,6 @@
           <t>Ekiti</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>/data/legislator_images/50.jpg?v=7</t>
@@ -2035,7 +1987,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>/data/legislator_images/51.jpg?v=7</t>
@@ -2066,7 +2017,6 @@
           <t>Cross River</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>/data/legislator_images/52.jpg?v=7</t>
@@ -2097,7 +2047,6 @@
           <t>Abia</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>/data/legislator_images/53.jpg?v=7</t>
@@ -2128,7 +2077,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>/data/legislator_images/54.jpg?v=7</t>
@@ -2159,7 +2107,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>/data/legislator_images/55.jpg?v=7</t>
@@ -2190,7 +2137,6 @@
           <t>Gombe</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>/data/legislator_images/56.jpg?v=7</t>
@@ -2221,7 +2167,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>/data/legislator_images/57.jpg?v=7</t>
@@ -2252,7 +2197,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>/data/legislator_images/58.jpg?v=7</t>
@@ -2283,7 +2227,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>/data/legislator_images/59.jpg?v=7</t>
@@ -2314,7 +2257,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>/data/legislator_images/60.jpg?v=7</t>
@@ -2345,7 +2287,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>/data/legislator_images/61.jpg?v=7</t>
@@ -2376,7 +2317,6 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>/data/legislator_images/62.jpg?v=7</t>
@@ -2407,7 +2347,6 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
           <t>/data/legislator_images/63.jpg?v=7</t>
@@ -2438,7 +2377,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
           <t>/data/legislator_images/64.jpg?v=7</t>
@@ -2469,7 +2407,6 @@
           <t>Abia</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>/data/legislator_images/65.jpg?v=7</t>
@@ -2500,7 +2437,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>/data/legislator_images/66.jpg?v=7</t>
@@ -2531,7 +2467,6 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
           <t>/data/legislator_images/67.jpg?v=7</t>
@@ -2562,7 +2497,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>/data/legislator_images/68.jpg?v=7</t>
@@ -2593,7 +2527,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>/data/legislator_images/69.jpg?v=7</t>
@@ -2624,7 +2557,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>/data/legislator_images/70.jpg?v=7</t>
@@ -2655,7 +2587,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>/data/legislator_images/71.jpg?v=7</t>
@@ -2686,7 +2617,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>/data/legislator_images/72.jpg?v=7</t>
@@ -2717,7 +2647,6 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>/data/legislator_images/73.jpg?v=7</t>
@@ -2748,7 +2677,6 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>/data/legislator_images/74.jpg?v=7</t>
@@ -2779,7 +2707,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>/data/legislator_images/75.jpg?v=7</t>
@@ -2810,7 +2737,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>/data/legislator_images/76.jpg?v=7</t>
@@ -2841,7 +2767,6 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>/data/legislator_images/77.jpg?v=7</t>
@@ -2872,7 +2797,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>/data/legislator_images/78.jpg?v=7</t>
@@ -2903,7 +2827,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>/data/legislator_images/79.jpg?v=7</t>
@@ -2934,7 +2857,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>/data/legislator_images/80.jpg?v=7</t>
@@ -2965,7 +2887,6 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
           <t>/data/legislator_images/81.jpg?v=7</t>
@@ -2996,7 +2917,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>/data/legislator_images/82.jpg?v=7</t>
@@ -3027,7 +2947,6 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>/data/legislator_images/83.jpg?v=7</t>
@@ -3058,7 +2977,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>/data/legislator_images/84.jpg?v=7</t>
@@ -3089,7 +3007,6 @@
           <t>Abia</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
           <t>/data/legislator_images/85.jpg?v=7</t>
@@ -3120,7 +3037,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>/data/legislator_images/86.jpg?v=7</t>
@@ -3151,7 +3067,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>/data/legislator_images/87.jpg?v=7</t>
@@ -3182,7 +3097,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>/data/legislator_images/88.jpg?v=7</t>
@@ -3213,7 +3127,6 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
           <t>/data/legislator_images/89.jpg?v=7</t>
@@ -3244,7 +3157,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>/data/legislator_images/90.jpg?v=7</t>
@@ -3275,7 +3187,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>/data/legislator_images/91.jpg?v=7</t>
@@ -3306,7 +3217,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
           <t>/data/legislator_images/92.jpg?v=7</t>
@@ -3337,7 +3247,6 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>/data/legislator_images/93.jpg?v=7</t>
@@ -3368,7 +3277,6 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>/data/legislator_images/94.jpg?v=7</t>
@@ -3399,7 +3307,6 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>/data/legislator_images/95.jpg?v=7</t>
@@ -3430,7 +3337,6 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>/data/legislator_images/96.jpg?v=7</t>
@@ -3461,7 +3367,6 @@
           <t>Abia</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>/data/legislator_images/97.jpg?v=7</t>
@@ -3492,7 +3397,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
           <t>/data/legislator_images/98.jpg?v=7</t>
@@ -3523,7 +3427,6 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>/data/legislator_images/99.jpg?v=7</t>
@@ -3554,7 +3457,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>/data/legislator_images/100.jpg?v=7</t>
@@ -3585,7 +3487,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>/data/legislator_images/101.jpg?v=7</t>
@@ -3616,7 +3517,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>/data/legislator_images/102.jpg?v=7</t>
@@ -3647,7 +3547,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>/data/legislator_images/103.jpg?v=7</t>
@@ -3678,7 +3577,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>/data/legislator_images/104.jpg?v=7</t>
@@ -3709,7 +3607,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>/data/legislator_images/105.jpg?v=7</t>
@@ -3740,7 +3637,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>/data/legislator_images/106.jpg?v=7</t>
@@ -3771,7 +3667,6 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>/data/legislator_images/107.jpg?v=7</t>
@@ -3802,7 +3697,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>/data/legislator_images/108.jpg?v=7</t>
@@ -3833,7 +3727,6 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>/data/legislator_images/109.jpg?v=7</t>
@@ -3864,7 +3757,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>/data/legislator_images/110.jpg?v=7</t>
@@ -3895,7 +3787,6 @@
           <t>Gombe</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>/data/legislator_images/111.jpg?v=7</t>
@@ -3926,7 +3817,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>/data/legislator_images/112.jpg?v=7</t>
@@ -3957,7 +3847,6 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
           <t>/data/legislator_images/113.jpg?v=7</t>
@@ -3988,7 +3877,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
           <t>/data/legislator_images/114.jpg?v=7</t>
@@ -4019,7 +3907,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>/data/legislator_images/115.jpg?v=7</t>
@@ -4050,7 +3937,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>/data/legislator_images/116.jpg?v=7</t>
@@ -4081,7 +3967,6 @@
           <t>Cross River</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
           <t>/data/legislator_images/117.jpg?v=7</t>
@@ -4112,7 +3997,6 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>/data/legislator_images/118.jpg?v=7</t>
@@ -4143,7 +4027,6 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
           <t>/data/legislator_images/119.jpg?v=7</t>
@@ -4174,7 +4057,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>/data/legislator_images/120.jpg?v=7</t>
@@ -4205,7 +4087,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>/data/legislator_images/121.jpg?v=7</t>
@@ -4236,7 +4117,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>/data/legislator_images/122.jpg?v=7</t>
@@ -4267,7 +4147,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>/data/legislator_images/123.jpg?v=7</t>
@@ -4298,7 +4177,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
           <t>/data/legislator_images/124.jpg?v=7</t>
@@ -4329,7 +4207,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>/data/legislator_images/125.jpg?v=7</t>
@@ -4360,7 +4237,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>/data/legislator_images/126.jpg?v=7</t>
@@ -4391,7 +4267,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
           <t>/data/legislator_images/127.jpg?v=7</t>
@@ -4457,7 +4332,6 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>/data/legislator_images/129.jpg?v=7</t>
@@ -4488,7 +4362,6 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>/data/legislator_images/130.jpg?v=7</t>
@@ -4519,7 +4392,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>/data/legislator_images/131.jpg?v=7</t>
@@ -4550,7 +4422,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
           <t>/data/legislator_images/132.jpg?v=7</t>
@@ -4686,7 +4557,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
           <t>/data/legislator_images/136.jpg?v=7</t>
@@ -4752,7 +4622,6 @@
           <t>Abia</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
           <t>/data/legislator_images/138.jpg?v=7</t>
@@ -4783,7 +4652,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
           <t>/data/legislator_images/139.jpg?v=7</t>
@@ -4849,7 +4717,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
           <t>/data/legislator_images/141.jpg?v=7</t>
@@ -4880,7 +4747,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
           <t>/data/legislator_images/142.jpg?v=7</t>
@@ -4911,7 +4777,6 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
           <t>/data/legislator_images/143.jpg?v=7</t>
@@ -4942,7 +4807,6 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
           <t>/data/legislator_images/144.jpg?v=7</t>
@@ -4973,7 +4837,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
           <t>/data/legislator_images/145.jpg?v=7</t>
@@ -5004,7 +4867,6 @@
           <t>Gombe</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
           <t>/data/legislator_images/146.jpg?v=7</t>
@@ -5035,7 +4897,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
         <is>
           <t>/data/legislator_images/147.jpg?v=7</t>
@@ -5101,7 +4962,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
           <t>/data/legislator_images/149.jpg?v=7</t>
@@ -5132,7 +4992,6 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
           <t>/data/legislator_images/150.jpg?v=7</t>
@@ -5163,7 +5022,6 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
           <t>/data/legislator_images/151.jpg?v=7</t>
@@ -5194,7 +5052,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
           <t>/data/legislator_images/152.jpg?v=7</t>
@@ -5225,7 +5082,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
           <t>/data/legislator_images/153.jpg?v=7</t>
@@ -5256,7 +5112,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
           <t>/data/legislator_images/154.jpg?v=7</t>
@@ -5287,7 +5142,6 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
           <t>/data/legislator_images/155.jpg?v=7</t>
@@ -5318,7 +5172,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
           <t>/data/legislator_images/156.jpg?v=7</t>
@@ -5349,7 +5202,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
           <t>/data/legislator_images/157.jpg?v=7</t>
@@ -5380,7 +5232,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
           <t>/data/legislator_images/158.jpg?v=7</t>
@@ -5411,7 +5262,6 @@
           <t>Cross River</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
           <t>/data/legislator_images/159.jpg?v=7</t>
@@ -5442,7 +5292,6 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
           <t>/data/legislator_images/160.jpg?v=7</t>
@@ -5473,7 +5322,6 @@
           <t>Federal Capital Territory</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
           <t>/data/legislator_images/161.jpg?v=7</t>
@@ -5504,7 +5352,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
           <t>/data/legislator_images/162.jpg?v=7</t>
@@ -5535,7 +5382,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
           <t>/data/legislator_images/163.jpg?v=7</t>
@@ -5566,7 +5412,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
           <t>/data/legislator_images/164.jpg?v=7</t>
@@ -5597,7 +5442,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
           <t>/data/legislator_images/165.jpg?v=7</t>
@@ -5628,7 +5472,6 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
           <t>/data/legislator_images/166.jpg?v=7</t>
@@ -5659,7 +5502,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
           <t>/data/legislator_images/167.jpg?v=7</t>
@@ -5690,7 +5532,6 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
           <t>/data/legislator_images/168.jpg?v=7</t>
@@ -5721,7 +5562,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
           <t>/data/legislator_images/169.jpg?v=7</t>
@@ -5752,7 +5592,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
           <t>/data/legislator_images/170.jpg?v=7</t>
@@ -5783,7 +5622,6 @@
           <t>Ekiti</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
           <t>/data/legislator_images/171.jpg?v=7</t>
@@ -5814,7 +5652,6 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
           <t>/data/legislator_images/172.jpg?v=7</t>
@@ -5845,7 +5682,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
           <t>/data/legislator_images/173.jpg?v=7</t>
@@ -5876,7 +5712,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
           <t>/data/legislator_images/174.jpg?v=7</t>
@@ -5907,7 +5742,6 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
           <t>/data/legislator_images/175.jpg?v=7</t>
@@ -5938,7 +5772,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
           <t>/data/legislator_images/176.jpg?v=7</t>
@@ -5969,7 +5802,6 @@
           <t>Cross River</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>/data/legislator_images/177.jpg?v=7</t>
@@ -6000,7 +5832,6 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
           <t>/data/legislator_images/178.jpg?v=7</t>
@@ -6031,7 +5862,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
           <t>/data/legislator_images/179.jpg?v=7</t>
@@ -6062,7 +5892,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
           <t>/data/legislator_images/180.jpg?v=7</t>
@@ -6093,7 +5922,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
           <t>/data/legislator_images/181.jpg?v=7</t>
@@ -6124,7 +5952,6 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>/data/legislator_images/182.jpg?v=7</t>
@@ -6155,7 +5982,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
           <t>/data/legislator_images/183.jpg?v=7</t>
@@ -6186,7 +6012,6 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
           <t>/data/legislator_images/184.jpg?v=7</t>
@@ -6217,7 +6042,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
           <t>/data/legislator_images/185.jpg?v=7</t>
@@ -6248,7 +6072,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
           <t>/data/legislator_images/186.jpg?v=7</t>
@@ -6279,7 +6102,6 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
           <t>/data/legislator_images/187.jpg?v=7</t>
@@ -6310,7 +6132,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
           <t>/data/legislator_images/188.jpg?v=7</t>
@@ -6341,7 +6162,6 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
           <t>/data/legislator_images/189.jpg?v=7</t>
@@ -6372,7 +6192,6 @@
           <t>Bayelsa</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
           <t>/data/legislator_images/190.jpg?v=7</t>
@@ -6403,7 +6222,6 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
           <t>/data/legislator_images/191.jpg?v=7</t>
@@ -6434,7 +6252,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
           <t>/data/legislator_images/192.jpg?v=7</t>
@@ -6465,7 +6282,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
           <t>/data/legislator_images/193.jpg?v=7</t>
@@ -6496,7 +6312,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
           <t>/data/legislator_images/194.jpg?v=7</t>
@@ -6527,7 +6342,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
           <t>/data/legislator_images/195.jpg?v=7</t>
@@ -6558,7 +6372,6 @@
           <t>Faskari/Kankara/Sabuwa</t>
         </is>
       </c>
-      <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
           <t>/data/legislator_images/196.jpg?v=7</t>
@@ -6589,7 +6402,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
           <t>/data/legislator_images/197.jpg?v=7</t>
@@ -6620,7 +6432,6 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
           <t>/data/legislator_images/198.jpg?v=7</t>
@@ -6651,7 +6462,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
           <t>/data/legislator_images/199.jpg?v=7</t>
@@ -6682,7 +6492,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
           <t>/data/legislator_images/200.jpg?v=7</t>
@@ -6713,7 +6522,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
           <t>/data/legislator_images/201.jpg?v=7</t>
@@ -6744,7 +6552,6 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
           <t>/data/legislator_images/202.jpg?v=7</t>
@@ -6775,7 +6582,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
           <t>/data/legislator_images/203.jpg?v=7</t>
@@ -6806,7 +6612,6 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
           <t>/data/legislator_images/204.jpg?v=7</t>
@@ -6837,7 +6642,6 @@
           <t>Abia</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
           <t>/data/legislator_images/205.jpg?v=7</t>
@@ -6868,7 +6672,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
           <t>/data/legislator_images/206.jpg?v=7</t>
@@ -6899,7 +6702,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
           <t>/data/legislator_images/207.jpg?v=7</t>
@@ -6930,7 +6732,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr">
         <is>
           <t>/data/legislator_images/208.jpg?v=7</t>
@@ -6961,7 +6762,6 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
           <t>/data/legislator_images/209.jpg?v=7</t>
@@ -6992,7 +6792,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F211" t="inlineStr"/>
       <c r="G211" t="inlineStr">
         <is>
           <t>/data/legislator_images/210.jpg?v=7</t>
@@ -7023,7 +6822,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr">
         <is>
           <t>/data/legislator_images/211.jpg?v=7</t>
@@ -7054,7 +6852,6 @@
           <t>Gombe</t>
         </is>
       </c>
-      <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
           <t>/data/legislator_images/212.jpg?v=7</t>
@@ -7085,7 +6882,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
           <t>/data/legislator_images/213.jpg?v=7</t>
@@ -7116,7 +6912,6 @@
           <t>Abia</t>
         </is>
       </c>
-      <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
           <t>/data/legislator_images/214.jpg?v=7</t>
@@ -7147,7 +6942,6 @@
           <t>Abia</t>
         </is>
       </c>
-      <c r="F216" t="inlineStr"/>
       <c r="G216" t="inlineStr">
         <is>
           <t>/data/legislator_images/215.jpg?v=7</t>
@@ -7178,7 +6972,6 @@
           <t>Cross River</t>
         </is>
       </c>
-      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>/data/legislator_images/216.jpg?v=7</t>
@@ -7209,7 +7002,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F218" t="inlineStr"/>
       <c r="G218" t="inlineStr">
         <is>
           <t>/data/legislator_images/217.jpg?v=7</t>
@@ -7240,7 +7032,6 @@
           <t>Ekiti</t>
         </is>
       </c>
-      <c r="F219" t="inlineStr"/>
       <c r="G219" t="inlineStr">
         <is>
           <t>/data/legislator_images/218.jpg?v=7</t>
@@ -7271,7 +7062,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr">
         <is>
           <t>/data/legislator_images/219.jpg?v=7</t>
@@ -7302,7 +7092,6 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="F221" t="inlineStr"/>
       <c r="G221" t="inlineStr">
         <is>
           <t>/data/legislator_images/220.jpg?v=7</t>
@@ -7333,7 +7122,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
           <t>/data/legislator_images/221.jpg?v=7</t>
@@ -7364,7 +7152,6 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="F223" t="inlineStr"/>
       <c r="G223" t="inlineStr">
         <is>
           <t>/data/legislator_images/222.jpg?v=7</t>
@@ -7395,7 +7182,6 @@
           <t>Ekiti</t>
         </is>
       </c>
-      <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr">
         <is>
           <t>/data/legislator_images/223.jpg?v=7</t>
@@ -7426,7 +7212,6 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr">
         <is>
           <t>/data/legislator_images/224.jpg?v=7</t>
@@ -7457,7 +7242,6 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="F226" t="inlineStr"/>
       <c r="G226" t="inlineStr">
         <is>
           <t>/data/legislator_images/225.jpg?v=7</t>
@@ -7488,7 +7272,6 @@
           <t>Ekiti</t>
         </is>
       </c>
-      <c r="F227" t="inlineStr"/>
       <c r="G227" t="inlineStr">
         <is>
           <t>/data/legislator_images/226.jpg?v=7</t>
@@ -7519,7 +7302,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
           <t>/data/legislator_images/227.jpg?v=7</t>
@@ -7550,7 +7332,6 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr">
         <is>
           <t>/data/legislator_images/228.jpg?v=7</t>
@@ -7581,7 +7362,6 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr">
         <is>
           <t>/data/legislator_images/229.jpg?v=7</t>
@@ -7609,10 +7389,9 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F231" t="inlineStr"/>
+          <t>Imo</t>
+        </is>
+      </c>
       <c r="G231" t="inlineStr">
         <is>
           <t>/data/legislator_images/230.jpg?v=7</t>
@@ -7643,7 +7422,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>/data/legislator_images/231.jpg?v=7</t>
@@ -7674,7 +7452,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr">
         <is>
           <t>/data/legislator_images/232.jpg?v=7</t>
@@ -7705,7 +7482,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
           <t>/data/legislator_images/233.jpg?v=7</t>
@@ -7736,7 +7512,6 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
           <t>/data/legislator_images/234.jpg?v=7</t>
@@ -7767,7 +7542,6 @@
           <t>Cross River</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>/data/legislator_images/235.jpg?v=7</t>
@@ -7798,7 +7572,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
           <t>/data/legislator_images/236.jpg?v=7</t>
@@ -7829,7 +7602,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
           <t>/data/legislator_images/237.jpg?v=7</t>
@@ -7860,7 +7632,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>/data/legislator_images/238.jpg?v=7</t>
@@ -7891,7 +7662,6 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>/data/legislator_images/239.jpg?v=7</t>
@@ -7922,7 +7692,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
           <t>/data/legislator_images/240.jpg?v=7</t>
@@ -7953,7 +7722,6 @@
           <t>Bayelsa</t>
         </is>
       </c>
-      <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
           <t>/data/legislator_images/241.jpg?v=7</t>
@@ -7984,7 +7752,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
           <t>/data/legislator_images/242.jpg?v=7</t>
@@ -8015,7 +7782,6 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
           <t>/data/legislator_images/243.jpg?v=7</t>
@@ -8046,7 +7812,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
           <t>/data/legislator_images/244.jpg?v=7</t>
@@ -8077,7 +7842,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
           <t>/data/legislator_images/245.jpg?v=7</t>
@@ -8108,7 +7872,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
           <t>/data/legislator_images/246.jpg?v=7</t>
@@ -8139,7 +7902,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
           <t>/data/legislator_images/247.jpg?v=7</t>
@@ -8170,7 +7932,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
           <t>/data/legislator_images/248.jpg?v=7</t>
@@ -8201,7 +7962,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
           <t>/data/legislator_images/249.jpg?v=7</t>
@@ -8232,7 +7992,6 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
           <t>/data/legislator_images/250.jpg?v=7</t>
@@ -8263,7 +8022,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
           <t>/data/legislator_images/251.jpg?v=7</t>
@@ -8294,7 +8052,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
           <t>/data/legislator_images/252.jpg?v=7</t>
@@ -8325,7 +8082,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
           <t>/data/legislator_images/253.jpg?v=7</t>
@@ -8356,7 +8112,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
           <t>/data/legislator_images/254.jpg?v=7</t>
@@ -8387,7 +8142,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
           <t>/data/legislator_images/255.jpg?v=7</t>
@@ -8418,7 +8172,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
           <t>/data/legislator_images/256.jpg?v=7</t>
@@ -8449,7 +8202,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
           <t>/data/legislator_images/257.jpg?v=7</t>
@@ -8480,7 +8232,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
           <t>/data/legislator_images/258.jpg?v=7</t>
@@ -8511,7 +8262,6 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
           <t>/data/legislator_images/259.jpg?v=7</t>
@@ -8542,7 +8292,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
           <t>/data/legislator_images/260.jpg?v=7</t>
@@ -8573,7 +8322,6 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
           <t>/data/legislator_images/261.jpg?v=7</t>
@@ -8604,7 +8352,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
           <t>/data/legislator_images/262.jpg?v=7</t>
@@ -8635,7 +8382,6 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
           <t>/data/legislator_images/263.jpg?v=7</t>
@@ -8666,7 +8412,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
           <t>/data/legislator_images/264.jpg?v=7</t>
@@ -8697,7 +8442,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
           <t>/data/legislator_images/265.jpg?v=7</t>
@@ -8728,7 +8472,6 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
           <t>/data/legislator_images/266.jpg?v=7</t>
@@ -8759,7 +8502,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
           <t>/data/legislator_images/267.jpg?v=7</t>
@@ -8790,7 +8532,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
           <t>/data/legislator_images/268.jpg?v=7</t>
@@ -8821,7 +8562,6 @@
           <t>Benue</t>
         </is>
       </c>
-      <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
           <t>/data/legislator_images/269.jpg?v=7</t>
@@ -8852,7 +8592,6 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
         <is>
           <t>/data/legislator_images/270.jpg?v=7</t>
@@ -8883,7 +8622,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
           <t>/data/legislator_images/271.jpg?v=7</t>
@@ -8914,7 +8652,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
           <t>/data/legislator_images/272.jpg?v=7</t>
@@ -8945,7 +8682,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
           <t>/data/legislator_images/273.jpg?v=7</t>
@@ -8976,7 +8712,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
           <t>/data/legislator_images/274.jpg?v=7</t>
@@ -9007,7 +8742,6 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
           <t>/data/legislator_images/275.jpg?v=7</t>
@@ -9038,7 +8772,6 @@
           <t>Akwa Ibom</t>
         </is>
       </c>
-      <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
           <t>/data/legislator_images/276.jpg?v=7</t>
@@ -9069,7 +8802,6 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
           <t>/data/legislator_images/277.jpg?v=7</t>
@@ -9100,7 +8832,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr">
         <is>
           <t>/data/legislator_images/278.jpg?v=7</t>
@@ -9131,7 +8862,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
           <t>/data/legislator_images/279.jpg?v=7</t>
@@ -9162,7 +8892,6 @@
           <t>Cross River</t>
         </is>
       </c>
-      <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
           <t>/data/legislator_images/280.jpg?v=7</t>
@@ -9193,7 +8922,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
           <t>/data/legislator_images/281.jpg?v=7</t>
@@ -9224,7 +8952,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>/data/legislator_images/282.jpg?v=7</t>
@@ -9255,7 +8982,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
           <t>/data/legislator_images/283.jpg?v=7</t>
@@ -9286,7 +9012,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
           <t>/data/legislator_images/284.jpg?v=7</t>
@@ -9317,7 +9042,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
         <is>
           <t>/data/legislator_images/285.jpg?v=7</t>
@@ -9348,7 +9072,6 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
           <t>/data/legislator_images/286.jpg?v=7</t>
@@ -9379,7 +9102,6 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
           <t>/data/legislator_images/287.jpg?v=7</t>
@@ -9410,7 +9132,6 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
           <t>/data/legislator_images/288.jpg?v=7</t>
@@ -9441,7 +9162,6 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
           <t>/data/legislator_images/289.jpg?v=7</t>
@@ -9472,7 +9192,6 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
           <t>/data/legislator_images/290.jpg?v=7</t>
@@ -9503,7 +9222,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
           <t>/data/legislator_images/291.jpg?v=7</t>
@@ -9534,7 +9252,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
           <t>/data/legislator_images/292.jpg?v=7</t>
@@ -9600,7 +9317,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
           <t>/data/legislator_images/294.jpg?v=7</t>
@@ -9631,7 +9347,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
           <t>/data/legislator_images/295.jpg?v=7</t>
@@ -9662,7 +9377,6 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
           <t>/data/legislator_images/296.jpg?v=7</t>
@@ -9728,7 +9442,6 @@
           <t>Bayelsa</t>
         </is>
       </c>
-      <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
           <t>/data/legislator_images/298.jpg?v=7</t>
@@ -9759,7 +9472,6 @@
           <t>Bayelsa</t>
         </is>
       </c>
-      <c r="F300" t="inlineStr"/>
       <c r="G300" t="inlineStr">
         <is>
           <t>/data/legislator_images/299.jpg?v=7</t>
@@ -9825,7 +9537,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F302" t="inlineStr"/>
       <c r="G302" t="inlineStr">
         <is>
           <t>/data/legislator_images/301.jpg?v=7</t>
@@ -9856,7 +9567,6 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="F303" t="inlineStr"/>
       <c r="G303" t="inlineStr">
         <is>
           <t>/data/legislator_images/302.jpg?v=7</t>
@@ -9887,7 +9597,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F304" t="inlineStr"/>
       <c r="G304" t="inlineStr">
         <is>
           <t>/data/legislator_images/303.jpg?v=7</t>
@@ -9918,7 +9627,6 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="F305" t="inlineStr"/>
       <c r="G305" t="inlineStr">
         <is>
           <t>/data/legislator_images/304.jpg?v=7</t>
@@ -9949,7 +9657,6 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="F306" t="inlineStr"/>
       <c r="G306" t="inlineStr">
         <is>
           <t>/data/legislator_images/305.jpg?v=7</t>
@@ -9980,7 +9687,6 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="F307" t="inlineStr"/>
       <c r="G307" t="inlineStr">
         <is>
           <t>/data/legislator_images/306.jpg?v=7</t>
@@ -10011,7 +9717,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="F308" t="inlineStr"/>
       <c r="G308" t="inlineStr">
         <is>
           <t>/data/legislator_images/307.jpg?v=7</t>
@@ -10042,7 +9747,6 @@
           <t>Ekiti</t>
         </is>
       </c>
-      <c r="F309" t="inlineStr"/>
       <c r="G309" t="inlineStr">
         <is>
           <t>/data/legislator_images/308.jpg?v=7</t>
@@ -10073,7 +9777,6 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="F310" t="inlineStr"/>
       <c r="G310" t="inlineStr">
         <is>
           <t>/data/legislator_images/309.jpg?v=7</t>
@@ -10104,7 +9807,6 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="F311" t="inlineStr"/>
       <c r="G311" t="inlineStr">
         <is>
           <t>/data/legislator_images/310.jpg?v=7</t>
@@ -10135,7 +9837,6 @@
           <t>Gombe</t>
         </is>
       </c>
-      <c r="F312" t="inlineStr"/>
       <c r="G312" t="inlineStr">
         <is>
           <t>/data/legislator_images/311.jpg?v=7</t>
@@ -10166,7 +9867,6 @@
           <t>Gombe</t>
         </is>
       </c>
-      <c r="F313" t="inlineStr"/>
       <c r="G313" t="inlineStr">
         <is>
           <t>/data/legislator_images/312.jpg?v=7</t>
@@ -10197,7 +9897,6 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="F314" t="inlineStr"/>
       <c r="G314" t="inlineStr">
         <is>
           <t>/data/legislator_images/313.jpg?v=7</t>
@@ -10228,7 +9927,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F315" t="inlineStr"/>
       <c r="G315" t="inlineStr">
         <is>
           <t>/data/legislator_images/314.jpg?v=7</t>
@@ -10259,7 +9957,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F316" t="inlineStr"/>
       <c r="G316" t="inlineStr">
         <is>
           <t>/data/legislator_images/315.jpg?v=7</t>
@@ -10290,7 +9987,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F317" t="inlineStr"/>
       <c r="G317" t="inlineStr">
         <is>
           <t>/data/legislator_images/316.jpg?v=7</t>
@@ -10321,7 +10017,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F318" t="inlineStr"/>
       <c r="G318" t="inlineStr">
         <is>
           <t>/data/legislator_images/317.jpg?v=7</t>
@@ -10387,7 +10082,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F320" t="inlineStr"/>
       <c r="G320" t="inlineStr">
         <is>
           <t>/data/legislator_images/319.jpg?v=7</t>
@@ -10418,7 +10112,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F321" t="inlineStr"/>
       <c r="G321" t="inlineStr">
         <is>
           <t>/data/legislator_images/320.jpg?v=7</t>
@@ -10449,7 +10142,6 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="F322" t="inlineStr"/>
       <c r="G322" t="inlineStr">
         <is>
           <t>/data/legislator_images/321.jpg?v=7</t>
@@ -10480,7 +10172,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F323" t="inlineStr"/>
       <c r="G323" t="inlineStr">
         <is>
           <t>/data/legislator_images/322.jpg?v=7</t>
@@ -10511,7 +10202,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F324" t="inlineStr"/>
       <c r="G324" t="inlineStr">
         <is>
           <t>/data/legislator_images/323.jpg?v=7</t>
@@ -10542,7 +10232,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F325" t="inlineStr"/>
       <c r="G325" t="inlineStr">
         <is>
           <t>/data/legislator_images/324.jpg?v=7</t>
@@ -10573,7 +10262,6 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="F326" t="inlineStr"/>
       <c r="G326" t="inlineStr">
         <is>
           <t>/data/legislator_images/325.jpg?v=7</t>
@@ -10604,7 +10292,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F327" t="inlineStr"/>
       <c r="G327" t="inlineStr">
         <is>
           <t>/data/legislator_images/326.jpg?v=7</t>
@@ -10635,7 +10322,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F328" t="inlineStr"/>
       <c r="G328" t="inlineStr">
         <is>
           <t>/data/legislator_images/327.jpg?v=7</t>
@@ -10666,7 +10352,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F329" t="inlineStr"/>
       <c r="G329" t="inlineStr">
         <is>
           <t>/data/legislator_images/328.jpg?v=7</t>
@@ -10697,7 +10382,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F330" t="inlineStr"/>
       <c r="G330" t="inlineStr">
         <is>
           <t>/data/legislator_images/329.jpg?v=7</t>
@@ -10728,7 +10412,6 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="F331" t="inlineStr"/>
       <c r="G331" t="inlineStr">
         <is>
           <t>/data/legislator_images/330.jpg?v=7</t>
@@ -10759,7 +10442,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F332" t="inlineStr"/>
       <c r="G332" t="inlineStr">
         <is>
           <t>/data/legislator_images/331.jpg?v=7</t>
@@ -10790,7 +10472,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F333" t="inlineStr"/>
       <c r="G333" t="inlineStr">
         <is>
           <t>/data/legislator_images/332.jpg?v=7</t>
@@ -10821,7 +10502,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F334" t="inlineStr"/>
       <c r="G334" t="inlineStr">
         <is>
           <t>/data/legislator_images/333.jpg?v=7</t>
@@ -10852,7 +10532,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr">
         <is>
           <t>/data/legislator_images/334.jpg?v=7</t>
@@ -10883,7 +10562,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr">
         <is>
           <t>/data/legislator_images/335.jpg?v=7</t>
@@ -10914,7 +10592,6 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr"/>
       <c r="G337" t="inlineStr">
         <is>
           <t>/data/legislator_images/336.jpg?v=7</t>
@@ -10945,7 +10622,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
           <t>/data/legislator_images/337.jpg?v=7</t>
@@ -10976,7 +10652,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
           <t>/data/legislator_images/338.jpg?v=7</t>
@@ -11007,7 +10682,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F340" t="inlineStr"/>
       <c r="G340" t="inlineStr">
         <is>
           <t>/data/legislator_images/339.jpg?v=7</t>
@@ -11038,7 +10712,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
           <t>/data/legislator_images/340.jpg?v=7</t>
@@ -11069,7 +10742,6 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr"/>
       <c r="G342" t="inlineStr">
         <is>
           <t>/data/legislator_images/341.jpg?v=7</t>
@@ -11100,7 +10772,6 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr">
         <is>
           <t>/data/legislator_images/342.jpg?v=7</t>
@@ -11131,7 +10802,6 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="F344" t="inlineStr"/>
       <c r="G344" t="inlineStr">
         <is>
           <t>/data/legislator_images/343.jpg?v=7</t>
@@ -11162,7 +10832,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F345" t="inlineStr"/>
       <c r="G345" t="inlineStr">
         <is>
           <t>/data/legislator_images/344.jpg?v=7</t>
@@ -11193,7 +10862,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F346" t="inlineStr"/>
       <c r="G346" t="inlineStr">
         <is>
           <t>/data/legislator_images/345.jpg?v=7</t>
@@ -11224,7 +10892,6 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="F347" t="inlineStr"/>
       <c r="G347" t="inlineStr">
         <is>
           <t>/data/legislator_images/346.jpg?v=7</t>
@@ -11255,7 +10922,6 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="F348" t="inlineStr"/>
       <c r="G348" t="inlineStr">
         <is>
           <t>/data/legislator_images/347.jpg?v=7</t>
@@ -11286,7 +10952,6 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="F349" t="inlineStr"/>
       <c r="G349" t="inlineStr">
         <is>
           <t>/data/legislator_images/348.jpg?v=7</t>
@@ -11317,7 +10982,6 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="F350" t="inlineStr"/>
       <c r="G350" t="inlineStr">
         <is>
           <t>/data/legislator_images/349.jpg?v=7</t>
@@ -11348,7 +11012,6 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="F351" t="inlineStr"/>
       <c r="G351" t="inlineStr">
         <is>
           <t>/data/legislator_images/350.jpg?v=7</t>
@@ -11379,7 +11042,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>/data/legislator_images/351.jpg?v=7</t>
@@ -11410,7 +11072,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F353" t="inlineStr"/>
       <c r="G353" t="inlineStr">
         <is>
           <t>/data/legislator_images/352.jpg?v=7</t>
@@ -11441,7 +11102,6 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
           <t>/data/legislator_images/353.jpg?v=7</t>
@@ -11472,7 +11132,6 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
           <t>/data/legislator_images/354.jpg?v=7</t>
@@ -11503,7 +11162,6 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="F356" t="inlineStr"/>
       <c r="G356" t="inlineStr">
         <is>
           <t>/data/legislator_images/355.jpg?v=7</t>
@@ -11534,7 +11192,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr">
         <is>
           <t>/data/legislator_images/356.jpg?v=7</t>
@@ -11565,7 +11222,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F358" t="inlineStr"/>
       <c r="G358" t="inlineStr">
         <is>
           <t>/data/legislator_images/357.jpg?v=7</t>
@@ -11596,7 +11252,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr">
         <is>
           <t>/data/legislator_images/358.jpg?v=7</t>
@@ -11627,7 +11282,6 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="F360" t="inlineStr"/>
       <c r="G360" t="inlineStr">
         <is>
           <t>/data/legislator_images/359.jpg?v=7</t>
@@ -11658,7 +11312,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F361" t="inlineStr"/>
       <c r="G361" t="inlineStr">
         <is>
           <t>/data/legislator_images/360.jpg?v=7</t>
@@ -11689,7 +11342,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F362" t="inlineStr"/>
       <c r="G362" t="inlineStr">
         <is>
           <t>/data/legislator_images/361.jpg?v=7</t>
@@ -11720,7 +11372,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F363" t="inlineStr"/>
       <c r="G363" t="inlineStr">
         <is>
           <t>/data/legislator_images/362.jpg?v=7</t>
@@ -11751,7 +11402,6 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="F364" t="inlineStr"/>
       <c r="G364" t="inlineStr">
         <is>
           <t>/data/legislator_images/363.jpg?v=7</t>
@@ -11782,7 +11432,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F365" t="inlineStr"/>
       <c r="G365" t="inlineStr">
         <is>
           <t>/data/legislator_images/364.jpg?v=7</t>
@@ -11813,7 +11462,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F366" t="inlineStr"/>
       <c r="G366" t="inlineStr">
         <is>
           <t>/data/legislator_images/365.jpg?v=7</t>
@@ -11844,7 +11492,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F367" t="inlineStr"/>
       <c r="G367" t="inlineStr">
         <is>
           <t>/data/legislator_images/366.jpg?v=7</t>
@@ -11910,7 +11557,6 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="F369" t="inlineStr"/>
       <c r="G369" t="inlineStr">
         <is>
           <t>/data/legislator_images/368.jpg?v=7</t>
@@ -11941,7 +11587,6 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="F370" t="inlineStr"/>
       <c r="G370" t="inlineStr">
         <is>
           <t>/data/legislator_images/369.jpg?v=7</t>
@@ -11972,7 +11617,6 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="F371" t="inlineStr"/>
       <c r="G371" t="inlineStr">
         <is>
           <t>/data/legislator_images/370.jpg?v=7</t>
@@ -12003,7 +11647,6 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="F372" t="inlineStr"/>
       <c r="G372" t="inlineStr">
         <is>
           <t>/data/legislator_images/371.jpg?v=7</t>
@@ -12034,7 +11677,6 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="F373" t="inlineStr"/>
       <c r="G373" t="inlineStr">
         <is>
           <t>/data/legislator_images/372.jpg?v=7</t>
@@ -12065,7 +11707,6 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="F374" t="inlineStr"/>
       <c r="G374" t="inlineStr">
         <is>
           <t>/data/legislator_images/373.jpg?v=7</t>
@@ -12096,7 +11737,6 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="F375" t="inlineStr"/>
       <c r="G375" t="inlineStr">
         <is>
           <t>/data/legislator_images/374.jpg?v=7</t>
@@ -12127,7 +11767,6 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="F376" t="inlineStr"/>
       <c r="G376" t="inlineStr">
         <is>
           <t>/data/legislator_images/375.jpg?v=7</t>

</xml_diff>

<commit_message>
Refresh 10th Assembly roster: 2026 party defections, AI studio photos, repo cleanup
- Party refresh for all members (PLAC API + web-researched 2025-2026 defections via PARTY_OVERRIDES); only Vacant has no party
- Rebuilt legislator photos as slug files (sen_*/rep_*), added missing photos, removed legacy numbered sets (984 files)
- AI-cleaned all 492 photos: rembg u2netp matting, white studio canvas, 22% headroom, 400x400 HD (clean_images_ai.py)
- Added ?v=4 image cache-buster; added rembg/onnxruntime to requirements
- Deleted obsolete one-off scripts; added README.md
</commit_message>
<xml_diff>
--- a/data/house_of_reps_master_final.xlsx
+++ b/data/house_of_reps_master_final.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,7 +479,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>/data/legislator_images/1.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abass_adekunle_adeogun.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>/data/legislator_images/2.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abdulhakeem_kamilu_ado.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -537,11 +537,7 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/3.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -567,11 +563,7 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/4.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -597,11 +589,7 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/5.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -627,11 +615,7 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/6.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -657,11 +641,7 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/7.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -689,7 +669,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>/data/legislator_images/8.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abdulrahman_ajiya.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -719,7 +699,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>/data/legislator_images/9.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abdussamad_ibrahim_dasuki.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -749,7 +729,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>/data/legislator_images/10.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abiodun_isiaq_akinlade.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -779,7 +759,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>/data/legislator_images/11.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abiodun_james_faleke.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -807,11 +787,7 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/12.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -837,11 +813,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/13.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -867,11 +839,7 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/14.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -899,7 +867,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>/data/legislator_images/15.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abubakar_yahaya_kusada.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -929,7 +897,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>/data/legislator_images/16.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adamu_hashimu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -959,7 +927,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>/data/legislator_images/17.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adamu_ibrahim_gamawa.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -987,11 +955,7 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/18.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1019,7 +983,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>/data/legislator_images/19.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adebayo_olusegun_balogun.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1013,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>/data/legislator_images/20.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adeboye_paul_kalajaiye.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1043,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>/data/legislator_images/21.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adedayo_samuel_adesola.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1107,11 +1071,7 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/22.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1137,11 +1097,7 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/23.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1169,7 +1125,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>/data/legislator_images/24.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adesola_ayoola_elegbeji.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1155,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>/data/legislator_images/25.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adetola_kafilat_ogbara.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1185,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>/data/legislator_images/26.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adetunji_abidemi_olusoji.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1262,11 +1218,7 @@
           <t>Cleaned &amp; Upscaled</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/27.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1294,7 +1246,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>/data/legislator_images/28.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adewunmi_oriyomi_onanuga.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1322,11 +1274,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/29.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1352,11 +1300,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/30.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1382,11 +1326,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/31.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1414,7 +1354,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>/data/legislator_images/32.jpg?v=7</t>
+          <t>/data/legislator_images/rep_afam_ogene.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1447,11 +1387,7 @@
           <t>Cleaned &amp; Upscaled</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/33.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1479,7 +1415,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>/data/legislator_images/34.jpg?v=7</t>
+          <t>/data/legislator_images/rep_agbedi_yeitiemone_frederick.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1507,11 +1443,7 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/35.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1539,7 +1471,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>/data/legislator_images/36.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ahmadu_usman_jaha.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1567,11 +1499,7 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/37.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1597,11 +1525,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/38.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1629,7 +1553,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>/data/legislator_images/39.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ahmed_idris_wase.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1583,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>/data/legislator_images/40.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ahmed_munir.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1613,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>/data/legislator_images/41.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ahmed_yinka_aluko.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1643,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>/data/legislator_images/42.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ajilo_umar.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1747,11 +1671,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/43.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1779,7 +1699,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>/data/legislator_images/44.jpg?v=7</t>
+          <t>/data/legislator_images/rep_akanni_clement_ademola.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1807,11 +1727,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/45.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1839,7 +1755,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>/data/legislator_images/46.jpg?v=7</t>
+          <t>/data/legislator_images/rep_akarachi_etinosa_tosan.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1785,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>/data/legislator_images/47.jpg?v=7</t>
+          <t>/data/legislator_images/rep_akiba_bassey_ekpenyong.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1815,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>/data/legislator_images/48.jpg?v=7</t>
+          <t>/data/legislator_images/rep_akingbaso_festus_olanrewaju.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1927,11 +1843,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/49.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1959,7 +1871,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>/data/legislator_images/50.jpg?v=7</t>
+          <t>/data/legislator_images/rep_akintunde_rotimi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1901,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>/data/legislator_images/51.jpg?v=7</t>
+          <t>/data/legislator_images/rep_akpatason_ohiozojeh_peter.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2019,7 +1931,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>/data/legislator_images/52.jpg?v=7</t>
+          <t>/data/legislator_images/rep_alex_egbona.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2049,7 +1961,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>/data/legislator_images/53.jpg?v=7</t>
+          <t>/data/legislator_images/rep_alexander_mascot_ikwechegh.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2079,7 +1991,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>/data/legislator_images/54.jpg?v=7</t>
+          <t>/data/legislator_images/rep_alhassan_ado_garba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2107,11 +2019,7 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/55.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2139,7 +2047,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>/data/legislator_images/56.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ali_isa.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2077,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>/data/legislator_images/57.jpg?v=7</t>
+          <t>/data/legislator_images/rep_aliu_ademorin_kuye.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2107,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>/data/legislator_images/58.jpg?v=7</t>
+          <t>/data/legislator_images/rep_aliyu_bappa_misau.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2227,11 +2135,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/59.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2259,7 +2163,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>/data/legislator_images/60.jpg?v=7</t>
+          <t>/data/legislator_images/rep_aliyu_mustapha_abdullahi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2287,11 +2191,7 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/61.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2319,7 +2219,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>/data/legislator_images/62.jpg?v=7</t>
+          <t>/data/legislator_images/rep_aliyu_wakili_boya.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2249,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>/data/legislator_images/63.jpg?v=7</t>
+          <t>/data/legislator_images/rep_aminu_jaji.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2377,11 +2277,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/64.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2409,7 +2305,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>/data/legislator_images/65.jpg?v=7</t>
+          <t>/data/legislator_images/rep_amobi_ogah.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2335,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>/data/legislator_images/66.jpg?v=7</t>
+          <t>/data/legislator_images/rep_amos_gwamna_magaji.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2365,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>/data/legislator_images/67.jpg?v=7</t>
+          <t>/data/legislator_images/rep_anayo_edwin_nwonu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2497,11 +2393,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/68.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2529,7 +2421,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>/data/legislator_images/69.jpg?v=7</t>
+          <t>/data/legislator_images/rep_austin_asema_achado.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2451,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>/data/legislator_images/70.jpg?v=7</t>
+          <t>/data/legislator_images/rep_auwalu_abdu_gwalabe.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2481,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>/data/legislator_images/71.jpg?v=7</t>
+          <t>/data/legislator_images/rep_awaji_inombek_dagomie_abiante.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2617,11 +2509,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/72.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2647,11 +2535,7 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/73.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2677,11 +2561,7 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/74.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2709,7 +2589,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>/data/legislator_images/75.jpg?v=7</t>
+          <t>/data/legislator_images/rep_babajimi_adegoke_benson.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2737,11 +2617,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/76.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2769,7 +2645,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>/data/legislator_images/77.jpg?v=7</t>
+          <t>/data/legislator_images/rep_bamidele_salam.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2675,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>/data/legislator_images/78.jpg?v=7</t>
+          <t>/data/legislator_images/rep_bashir_zubairu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2827,11 +2703,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/79.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2859,7 +2731,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>/data/legislator_images/80.jpg?v=7</t>
+          <t>/data/legislator_images/rep_bashiru_usman_gorau.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2889,7 +2761,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>/data/legislator_images/81.jpg?v=7</t>
+          <t>/data/legislator_images/rep_bello_a_kaoje.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -2917,11 +2789,7 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/82.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2947,11 +2815,7 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/83.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2977,11 +2841,7 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/84.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3009,7 +2869,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>/data/legislator_images/85.jpg?v=7</t>
+          <t>/data/legislator_images/rep_benjamin_kalu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3039,7 +2899,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>/data/legislator_images/86.jpg?v=7</t>
+          <t>/data/legislator_images/rep_billy_famous_osawaru.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3069,7 +2929,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>/data/legislator_images/87.jpg?v=7</t>
+          <t>/data/legislator_images/rep_blessing_chigeru_amadi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3099,7 +2959,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>/data/legislator_images/88.jpg?v=7</t>
+          <t>/data/legislator_images/rep_blessing_onyeche_onuh.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3129,7 +2989,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>/data/legislator_images/89.jpg?v=7</t>
+          <t>/data/legislator_images/rep_befford_onwuegbu_anayo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3019,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>/data/legislator_images/90.jpg?v=7</t>
+          <t>/data/legislator_images/rep_boma_goodhead.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3187,11 +3047,7 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/91.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3219,7 +3075,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>/data/legislator_images/92.jpg?v=7</t>
+          <t>/data/legislator_images/rep_bukar_talba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3249,7 +3105,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>/data/legislator_images/93.jpg?v=7</t>
+          <t>/data/legislator_images/rep_chike_john_okafor.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3135,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>/data/legislator_images/94.jpg?v=7</t>
+          <t>/data/legislator_images/rep_chimaobi_sam_atu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3307,11 +3163,7 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/95.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3339,7 +3191,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>/data/legislator_images/96.jpg?v=7</t>
+          <t>/data/legislator_images/rep_chinedu_tochukwu_okere.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3221,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>/data/legislator_images/97.jpg?v=7</t>
+          <t>/data/legislator_images/rep_chris_nkwonta.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3251,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>/data/legislator_images/98.jpg?v=7</t>
+          <t>/data/legislator_images/rep_clement_jimbo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3427,11 +3279,7 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/99.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3459,7 +3307,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>/data/legislator_images/100.jpg?v=7</t>
+          <t>/data/legislator_images/rep_cryril_hart_godwin.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3337,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>/data/legislator_images/101.jpg?v=7</t>
+          <t>/data/legislator_images/rep_dabo_ismaila_haruna.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3517,11 +3365,7 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/102.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -3549,7 +3393,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>/data/legislator_images/103.jpg?v=7</t>
+          <t>/data/legislator_images/rep_dalyop_chollom_fom.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3423,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>/data/legislator_images/104.jpg?v=7</t>
+          <t>/data/legislator_images/rep_daniel_asama_ago.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3453,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>/data/legislator_images/105.jpg?v=7</t>
+          <t>/data/legislator_images/rep_david_ogewu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3483,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>/data/legislator_images/106.jpg?v=7</t>
+          <t>/data/legislator_images/rep_dennis_idahosa.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3513,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>/data/legislator_images/107.jpg?v=7</t>
+          <t>/data/legislator_images/rep_dibiagwu_eugene_okechukwu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3543,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>/data/legislator_images/108.jpg?v=7</t>
+          <t>/data/legislator_images/rep_dominic_okafor.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3727,11 +3571,7 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/109.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -3757,11 +3597,7 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/110.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -3789,7 +3625,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>/data/legislator_images/111.jpg?v=7</t>
+          <t>/data/legislator_images/rep_el_rasheed_abdullahi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3819,7 +3655,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>/data/legislator_images/112.jpg?v=7</t>
+          <t>/data/legislator_images/rep_emeka_idu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3685,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>/data/legislator_images/113.jpg?v=7</t>
+          <t>/data/legislator_images/rep_emeka_martins_chinedu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3715,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>/data/legislator_images/114.jpg?v=7</t>
+          <t>/data/legislator_images/rep_emmanuel_effiong_ukpong_udo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3909,7 +3745,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>/data/legislator_images/115.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ereyitomi_thomas.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3775,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>/data/legislator_images/116.jpg?v=7</t>
+          <t>/data/legislator_images/rep_esosa_iyawe.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3969,7 +3805,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>/data/legislator_images/117.jpg?v=7</t>
+          <t>/data/legislator_images/rep_etaba_michael_irom.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3835,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>/data/legislator_images/118.jpg?v=7</t>
+          <t>/data/legislator_images/rep_eze_nwachukwu_eze.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4029,7 +3865,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>/data/legislator_images/119.jpg?v=7</t>
+          <t>/data/legislator_images/rep_fatima_talba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4059,7 +3895,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>/data/legislator_images/120.jpg?v=7</t>
+          <t>/data/legislator_images/rep_fidelis_joseph_bagudu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4089,7 +3925,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>/data/legislator_images/121.jpg?v=7</t>
+          <t>/data/legislator_images/rep_fola_oyekunle.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4119,7 +3955,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>/data/legislator_images/122.jpg?v=7</t>
+          <t>/data/legislator_images/rep_francis_ejiroghene_waive.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4149,7 +3985,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>/data/legislator_images/123.jpg?v=7</t>
+          <t>/data/legislator_images/rep_fuad_kayode_laguda.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4015,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>/data/legislator_images/124.jpg?v=7</t>
+          <t>/data/legislator_images/rep_gabriel_saleh_zock.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4045,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>/data/legislator_images/125.jpg?v=7</t>
+          <t>/data/legislator_images/rep_gagdi_adamu_yusuf.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4237,11 +4073,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/126.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -4269,7 +4101,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>/data/legislator_images/127.jpg?v=7</t>
+          <t>/data/legislator_images/rep_garba_ibrahim_muhammad.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4136,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>/data/legislator_images/128.jpg?v=7</t>
+          <t>/data/legislator_images/rep_garba_umar_uba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4166,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>/data/legislator_images/129.jpg?v=7</t>
+          <t>/data/legislator_images/rep_gaza_jonathan_gbefwi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4196,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>/data/legislator_images/130.jpg?v=7</t>
+          <t>/data/legislator_images/rep_gboyega_nasir_isiaka.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4392,11 +4224,7 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/131.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -4422,11 +4250,7 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/132.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -4459,7 +4283,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>/data/legislator_images/133.jpg?v=7</t>
+          <t>/data/legislator_images/rep_harrison_anozie_nwadike.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4318,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>/data/legislator_images/134.jpg?v=7</t>
+          <t>/data/legislator_images/rep_hassan_mohammed.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4353,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>/data/legislator_images/135.jpg?v=7</t>
+          <t>/data/legislator_images/rep_hassan_shehu_hussain.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4383,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>/data/legislator_images/136.jpg?v=7</t>
+          <t>/data/legislator_images/rep_henry_odianosen_okojie.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4592,11 +4416,7 @@
           <t>Cleaned &amp; Upscaled</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/137.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -4624,7 +4444,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>/data/legislator_images/138.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ibe_okwara_osonwa.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4652,11 +4472,7 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/139.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -4687,11 +4503,7 @@
           <t>Cleaned &amp; Upscaled</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/140.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -4719,7 +4531,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>/data/legislator_images/141.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ibrahim_hamisu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4747,11 +4559,7 @@
           <t>Borno</t>
         </is>
       </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/142.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -4779,7 +4587,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>/data/legislator_images/143.jpg?v=7</t>
+          <t>/data/legislator_images/rep_iduma_enwo_igariwey.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4809,7 +4617,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>/data/legislator_images/144.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ifeoluwa_ehindero.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4647,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>/data/legislator_images/145.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ime_bassey_okon.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4869,7 +4677,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>/data/legislator_images/146.jpg?v=7</t>
+          <t>/data/legislator_images/rep_inuwa_garba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4899,7 +4707,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>/data/legislator_images/147.jpg?v=7</t>
+          <t>/data/legislator_images/rep_isa_dogonyaro.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4742,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>/data/legislator_images/148.jpg?v=7</t>
+          <t>/data/legislator_images/rep_isa_mohammed_anka.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -4962,11 +4770,7 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/149.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -4994,7 +4798,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>/data/legislator_images/150.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ja_afar_abubakar_magaji.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5024,7 +4828,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>/data/legislator_images/151.jpg?v=7</t>
+          <t>/data/legislator_images/rep_jaafaru_yakubu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5054,7 +4858,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>/data/legislator_images/152.jpg?v=7</t>
+          <t>/data/legislator_images/rep_jafaru_gambo_leko.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5082,11 +4886,7 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/153.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -5114,7 +4914,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>/data/legislator_images/154.jpg?v=7</t>
+          <t>/data/legislator_images/rep_jalio_hussaini_mohammed.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5142,11 +4942,7 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/155.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -5174,7 +4970,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>/data/legislator_images/156.jpg?v=7</t>
+          <t>/data/legislator_images/rep_jesse_okey_joe_onuakachi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5204,7 +5000,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>/data/legislator_images/157.jpg?v=7</t>
+          <t>/data/legislator_images/rep_john_moenwul_dafaan.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5030,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>/data/legislator_images/158.jpg?v=7</t>
+          <t>/data/legislator_images/rep_jonathan_ajirioghene_ukodhiko.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5060,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>/data/legislator_images/159.jpg?v=7</t>
+          <t>/data/legislator_images/rep_joseph_bassey.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5292,11 +5088,7 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/160.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -5324,7 +5116,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>/data/legislator_images/161.jpg?v=7</t>
+          <t>/data/legislator_images/rep_joshua_chinedu_obika.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5352,11 +5144,7 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="G163" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/162.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -5384,7 +5172,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>/data/legislator_images/163.jpg?v=7</t>
+          <t>/data/legislator_images/rep_jubrin_abdulmumin.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5414,7 +5202,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>/data/legislator_images/164.jpg?v=7</t>
+          <t>/data/legislator_images/rep_julius_gbabojor_pondi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5232,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>/data/legislator_images/165.jpg?v=7</t>
+          <t>/data/legislator_images/rep_julius_ihonvbere.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5474,7 +5262,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>/data/legislator_images/166.jpg?v=7</t>
+          <t>/data/legislator_images/rep_kabir_tukura_ibrahim.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5504,7 +5292,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>/data/legislator_images/167.jpg?v=7</t>
+          <t>/data/legislator_images/rep_kabiru_alhassan_usman_rurum.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5532,11 +5320,7 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="G169" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/168.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -5564,7 +5348,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>/data/legislator_images/169.jpg?v=7</t>
+          <t>/data/legislator_images/rep_kelechi_nwogu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5594,7 +5378,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>/data/legislator_images/170.jpg?v=7</t>
+          <t>/data/legislator_images/rep_kingsley_chinda.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5624,7 +5408,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>/data/legislator_images/171.jpg?v=7</t>
+          <t>/data/legislator_images/rep_kolawole_davidson_akinlayo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5654,7 +5438,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>/data/legislator_images/172.jpg?v=7</t>
+          <t>/data/legislator_images/rep_kwamoti_bitrus_laori.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5684,7 +5468,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>/data/legislator_images/173.jpg?v=7</t>
+          <t>/data/legislator_images/rep_lalu_ishaya_david.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5712,11 +5496,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/174.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -5742,11 +5522,7 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/175.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -5774,7 +5550,7 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>/data/legislator_images/176.jpg?v=7</t>
+          <t>/data/legislator_images/rep_leke_joseph_abejide.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5804,7 +5580,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>/data/legislator_images/177.jpg?v=7</t>
+          <t>/data/legislator_images/rep_lemke_emil_inyang.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5832,11 +5608,7 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/178.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -5864,7 +5636,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>/data/legislator_images/179.jpg?v=7</t>
+          <t>/data/legislator_images/rep_makki_yalloman_abubakar.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5894,7 +5666,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>/data/legislator_images/180.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mallam_bukar_gana.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5696,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>/data/legislator_images/181.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mansur_manu_soro.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -5952,11 +5724,7 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/182.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -5984,7 +5752,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>/data/legislator_images/183.jpg?v=7</t>
+          <t>/data/legislator_images/rep_marcus_onobun.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6014,7 +5782,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>/data/legislator_images/184.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mark_chidi_obetta.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6044,7 +5812,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>/data/legislator_images/185.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mark_udo_esset.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6074,7 +5842,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>/data/legislator_images/186.jpg?v=7</t>
+          <t>/data/legislator_images/rep_martins_etim_esin.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6102,11 +5870,7 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="G188" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/187.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -6134,7 +5898,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>/data/legislator_images/188.jpg?v=7</t>
+          <t>/data/legislator_images/rep_midala_usman_balami.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6164,7 +5928,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>/data/legislator_images/189.jpg?v=7</t>
+          <t>/data/legislator_images/rep_miriam_onuoha.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6194,7 +5958,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>/data/legislator_images/190.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mitema_obordor.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6222,11 +5986,7 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/191.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -6254,7 +6014,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>/data/legislator_images/192.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mohammed_bello_el_rufai.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6284,7 +6044,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>/data/legislator_images/193.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mohammed_bello_shehu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6312,11 +6072,7 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="G195" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/194.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -6344,7 +6100,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>/data/legislator_images/195.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mohammed_dan_abba_shehu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6374,7 +6130,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>/data/legislator_images/196.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mohammed_jamilu_katsina.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6404,7 +6160,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>/data/legislator_images/197.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mohammed_saidu_bargaja.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6434,7 +6190,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>/data/legislator_images/198.jpg?v=7</t>
+          <t>/data/legislator_images/rep_morufu_adewale_adebayo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6464,7 +6220,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>/data/legislator_images/199.jpg?v=7</t>
+          <t>/data/legislator_images/rep_moses_oluwatoyin_fayinka.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6492,11 +6248,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G201" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/200.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -6524,7 +6276,7 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>/data/legislator_images/201.jpg?v=7</t>
+          <t>/data/legislator_images/rep_moshood_olanrewaju_oshun.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6552,11 +6304,7 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="G203" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/202.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -6584,7 +6332,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>/data/legislator_images/203.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mukhtar_umar_zakari.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6362,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>/data/legislator_images/204.jpg?v=7</t>
+          <t>/data/legislator_images/rep_muktar_tolani_shagaya.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6392,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>/data/legislator_images/205.jpg?v=7</t>
+          <t>/data/legislator_images/rep_munachim_alozie.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6674,7 +6422,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>/data/legislator_images/206.jpg?v=7</t>
+          <t>/data/legislator_images/rep_murphy_osaro_omoruyi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6704,7 +6452,7 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>/data/legislator_images/207.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ngozi_okolie.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6734,7 +6482,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>/data/legislator_images/208.jpg?v=7</t>
+          <t>/data/legislator_images/rep_nicholas_ebomo_mutu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6762,11 +6510,7 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="G210" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/209.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -6792,11 +6536,7 @@
           <t>Delta</t>
         </is>
       </c>
-      <c r="G211" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/210.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -6824,7 +6564,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>/data/legislator_images/211.jpg?v=7</t>
+          <t>/data/legislator_images/rep_nwaeke_felix_uche.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6854,7 +6594,7 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>/data/legislator_images/212.jpg?v=7</t>
+          <t>/data/legislator_images/rep_obeid_paul_shehu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6624,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>/data/legislator_images/213.jpg?v=7</t>
+          <t>/data/legislator_images/rep_obiageli_lillian_orogbu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6654,7 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>/data/legislator_images/214.jpg?v=7</t>
+          <t>/data/legislator_images/rep_obinna_aguocha.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6944,7 +6684,7 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>/data/legislator_images/215.jpg?v=7</t>
+          <t>/data/legislator_images/rep_obinna_ginger_onwusibe.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -6974,7 +6714,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>/data/legislator_images/216.jpg?v=7</t>
+          <t>/data/legislator_images/rep_offiono_godwin.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7004,7 +6744,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>/data/legislator_images/217.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ojema_ojotu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7034,7 +6774,7 @@
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>/data/legislator_images/218.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ojuawo_rufus_adeniyi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7064,7 +6804,7 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>/data/legislator_images/219.jpg?v=7</t>
+          <t>/data/legislator_images/rep_okpolupm_etteh.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7092,11 +6832,7 @@
           <t>Ondo</t>
         </is>
       </c>
-      <c r="G221" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/220.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -7122,11 +6858,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G222" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/221.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -7154,7 +6886,7 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>/data/legislator_images/222.jpg?v=7</t>
+          <t>/data/legislator_images/rep_olatunji_akinosi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7184,7 +6916,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>/data/legislator_images/223.jpg?v=7</t>
+          <t>/data/legislator_images/rep_olufemi_richard_bamisile.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7212,11 +6944,7 @@
           <t>Ogun</t>
         </is>
       </c>
-      <c r="G225" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/224.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -7244,7 +6972,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>/data/legislator_images/225.jpg?v=7</t>
+          <t>/data/legislator_images/rep_olumide_babatunde_osoba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7274,7 +7002,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>/data/legislator_images/226.jpg?v=7</t>
+          <t>/data/legislator_images/rep_olusola_steve_fatoba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7302,11 +7030,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G228" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/227.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -7334,7 +7058,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>/data/legislator_images/228.jpg?v=7</t>
+          <t>/data/legislator_images/rep_oluwole_oke.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7364,7 +7088,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>/data/legislator_images/229.jpg?v=7</t>
+          <t>/data/legislator_images/rep_osi_kama_nkemkanma.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7394,7 +7118,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>/data/legislator_images/230.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ozurigbo_ugonna.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7424,7 +7148,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>/data/legislator_images/231.jpg?v=7</t>
+          <t>/data/legislator_images/rep_pascal_agbodike.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7454,7 +7178,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>/data/legislator_images/232.jpg?v=7</t>
+          <t>/data/legislator_images/rep_patrick_umoh.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7484,7 +7208,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>/data/legislator_images/233.jpg?v=7</t>
+          <t>/data/legislator_images/rep_paul_asuquo_ekpo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7514,7 +7238,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>/data/legislator_images/234.jpg?v=7</t>
+          <t>/data/legislator_images/rep_paul_nnamchi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7542,11 +7266,7 @@
           <t>Cross River</t>
         </is>
       </c>
-      <c r="G236" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/235.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -7572,11 +7292,7 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="G237" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/236.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -7604,7 +7320,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>/data/legislator_images/237.jpg?v=7</t>
+          <t>/data/legislator_images/rep_philip_agbese.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7634,7 +7350,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>/data/legislator_images/238.jpg?v=7</t>
+          <t>/data/legislator_images/rep_prince_solomon_wombo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7664,7 +7380,7 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>/data/legislator_images/239.jpg?v=7</t>
+          <t>/data/legislator_images/rep_rabiu_garba_kamba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7694,7 +7410,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>/data/legislator_images/240.jpg?v=7</t>
+          <t>/data/legislator_images/rep_rabiu_yusuf.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7724,7 +7440,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>/data/legislator_images/241.jpg?v=7</t>
+          <t>/data/legislator_images/rep_rodney_ebikebina_ambiowei.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7752,11 +7468,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G243" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/242.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -7784,7 +7496,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>/data/legislator_images/243.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sadiq_abbas_tafida.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7814,7 +7526,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>/data/legislator_images/244.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sadiq_ango_abdullahi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7844,7 +7556,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>/data/legislator_images/245.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sagir_koki.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7872,11 +7584,7 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="G247" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/246.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -7902,11 +7610,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G248" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/247.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -7934,7 +7638,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>/data/legislator_images/248.jpg?v=7</t>
+          <t>/data/legislator_images/rep_salman_idris.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7964,7 +7668,7 @@
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>/data/legislator_images/249.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sani_adamu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -7992,11 +7696,7 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="G251" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/250.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -8024,7 +7724,7 @@
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>/data/legislator_images/251.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sani_umar_bala.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8054,7 +7754,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>/data/legislator_images/252.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sanni_abdulraheem.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8084,7 +7784,7 @@
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>/data/legislator_images/253.jpg?v=7</t>
+          <t>/data/legislator_images/rep_satomi_ahmad.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8114,7 +7814,7 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>/data/legislator_images/254.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sekav_dzua_iyortyom.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8142,11 +7842,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G256" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/255.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -8174,7 +7870,7 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>/data/legislator_images/256.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sesoo_ikpagher.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8204,7 +7900,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>/data/legislator_images/257.jpg?v=7</t>
+          <t>/data/legislator_images/rep_shehu_dalhatu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8234,7 +7930,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>/data/legislator_images/258.jpg?v=7</t>
+          <t>/data/legislator_images/rep_shehu_saleh_rijau.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8264,7 +7960,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>/data/legislator_images/259.jpg?v=7</t>
+          <t>/data/legislator_images/rep_simon_chukwuemeka_atigwe.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8294,7 +7990,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>/data/legislator_images/260.jpg?v=7</t>
+          <t>/data/legislator_images/rep_solomon_t_bob.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8322,11 +8018,7 @@
           <t>Zamfara</t>
         </is>
       </c>
-      <c r="G262" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/261.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -8354,7 +8046,7 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>/data/legislator_images/262.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sunday_anamero_dekeri.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8384,7 +8076,7 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>/data/legislator_images/263.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sunday_umeha.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8414,7 +8106,7 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>/data/legislator_images/264.jpg?v=7</t>
+          <t>/data/legislator_images/rep_tajudeen_abbas.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8442,11 +8134,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G266" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/265.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -8474,7 +8162,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>/data/legislator_images/266.jpg?v=7</t>
+          <t>/data/legislator_images/rep_taofeek_abimbola_ajilesoro.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8504,7 +8192,7 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>/data/legislator_images/267.jpg?v=7</t>
+          <t>/data/legislator_images/rep_tarkighir_dickson_dominic.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8532,11 +8220,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G269" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/268.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -8564,7 +8248,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>/data/legislator_images/269.jpg?v=7</t>
+          <t>/data/legislator_images/rep_terseer_ugbor.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8592,11 +8276,7 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/270.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -8622,11 +8302,7 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="G272" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/271.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -8654,7 +8330,7 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>/data/legislator_images/272.jpg?v=7</t>
+          <t>/data/legislator_images/rep_tolulope_tiwalola_akande_sadipe.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8684,7 +8360,7 @@
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>/data/legislator_images/273.jpg?v=7</t>
+          <t>/data/legislator_images/rep_uchenna_okonkwo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8714,7 +8390,7 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>/data/legislator_images/274.jpg?v=7</t>
+          <t>/data/legislator_images/rep_uduak_alphonsus_odudoh.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8744,7 +8420,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>/data/legislator_images/275.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ugochinyere_onyinye_ikeagwuonu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8774,7 +8450,7 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>/data/legislator_images/276.jpg?v=7</t>
+          <t>/data/legislator_images/rep_unyime_josiah_idem.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8804,7 +8480,7 @@
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>/data/legislator_images/277.jpg?v=7</t>
+          <t>/data/legislator_images/rep_useni_mark_bako.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8832,11 +8508,7 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="G279" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/278.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -8864,7 +8536,7 @@
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>/data/legislator_images/279.jpg?v=7</t>
+          <t>/data/legislator_images/rep_usman_zannah.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8894,7 +8566,7 @@
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>/data/legislator_images/280.jpg?v=7</t>
+          <t>/data/legislator_images/rep_victor_abang.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8924,7 +8596,7 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>/data/legislator_images/281.jpg?v=7</t>
+          <t>/data/legislator_images/rep_victor_obuzor.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -8952,11 +8624,7 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="G283" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/282.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -8984,7 +8652,7 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>/data/legislator_images/283.jpg?v=7</t>
+          <t>/data/legislator_images/rep_yusuf_datti.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9014,7 +8682,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>/data/legislator_images/284.jpg?v=7</t>
+          <t>/data/legislator_images/rep_yusuf_shitu_galambi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9044,7 +8712,7 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>/data/legislator_images/285.jpg?v=7</t>
+          <t>/data/legislator_images/rep_zainab_gimba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9074,7 +8742,7 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>/data/legislator_images/286.jpg?v=7</t>
+          <t>/data/legislator_images/rep_zakaria_dauda_nyampa.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9104,7 +8772,7 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>/data/legislator_images/287.jpg?v=7</t>
+          <t>/data/legislator_images/rep_james_barka.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9134,7 +8802,7 @@
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>/data/legislator_images/288.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mohammed_inuwa_bassi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9162,11 +8830,7 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="G290" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/289.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -9192,11 +8856,7 @@
           <t>Adamawa</t>
         </is>
       </c>
-      <c r="G291" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/290.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -9224,7 +8884,7 @@
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>/data/legislator_images/291.jpg?v=7</t>
+          <t>/data/legislator_images/rep_aniekwe_peter.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9254,7 +8914,7 @@
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t>/data/legislator_images/292.jpg?v=7</t>
+          <t>/data/legislator_images/rep_chinwe_nnabuife.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9287,11 +8947,7 @@
           <t>Cleaned &amp; Upscaled</t>
         </is>
       </c>
-      <c r="G294" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/293.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -9317,11 +8973,7 @@
           <t>Anambra</t>
         </is>
       </c>
-      <c r="G295" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/294.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -9349,7 +9001,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>/data/legislator_images/295.jpg?v=7</t>
+          <t>/data/legislator_images/rep_aliyu_aminu_garu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9377,11 +9029,7 @@
           <t>Bauchi</t>
         </is>
       </c>
-      <c r="G297" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/296.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -9414,7 +9062,7 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>/data/legislator_images/297.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sani_tanko.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9092,7 @@
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>/data/legislator_images/298.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ebikake_enenimiete.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9474,7 +9122,7 @@
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>/data/legislator_images/299.jpg?v=7</t>
+          <t>/data/legislator_images/rep_oboku_abonsizibe_oforji.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9507,11 +9155,7 @@
           <t>Cleaned &amp; Upscaled</t>
         </is>
       </c>
-      <c r="G301" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/300.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -9539,7 +9183,7 @@
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>/data/legislator_images/301.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abdulkadir_rahis.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9569,7 +9213,7 @@
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>/data/legislator_images/302.jpg?v=7</t>
+          <t>/data/legislator_images/rep_muktar_aliyu_betara.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9599,7 +9243,7 @@
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>/data/legislator_images/303.jpg?v=7</t>
+          <t>/data/legislator_images/rep_victor_nwokolo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9629,7 +9273,7 @@
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>/data/legislator_images/304.jpg?v=7</t>
+          <t>/data/legislator_images/rep_erhiatake_ibori_suenu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9657,11 +9301,7 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="G306" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/305.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -9687,11 +9327,7 @@
           <t>Ebonyi</t>
         </is>
       </c>
-      <c r="G307" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/306.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -9717,11 +9353,7 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="G308" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/307.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -9747,11 +9379,7 @@
           <t>Ekiti</t>
         </is>
       </c>
-      <c r="G309" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/308.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -9777,11 +9405,7 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="G310" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/309.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -9807,11 +9431,7 @@
           <t>Enugu</t>
         </is>
       </c>
-      <c r="G311" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/310.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -9839,7 +9459,7 @@
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>/data/legislator_images/311.jpg?v=7</t>
+          <t>/data/legislator_images/rep_usman_bello_kumo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9869,7 +9489,7 @@
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>/data/legislator_images/312.jpg?v=7</t>
+          <t>/data/legislator_images/rep_yaya_bauchi_tongo.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9897,11 +9517,7 @@
           <t>Imo</t>
         </is>
       </c>
-      <c r="G314" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/313.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -9927,11 +9543,7 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="G315" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/314.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -9959,7 +9571,7 @@
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t>/data/legislator_images/315.jpg?v=7</t>
+          <t>/data/legislator_images/rep_adamu_yakubu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -9989,7 +9601,7 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>/data/legislator_images/316.jpg?v=7</t>
+          <t>/data/legislator_images/rep_muktar_muhhammad.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10019,7 +9631,7 @@
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>/data/legislator_images/317.jpg?v=7</t>
+          <t>/data/legislator_images/rep_fulata_hassan.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10052,11 +9664,7 @@
           <t>Cleaned &amp; Upscaled</t>
         </is>
       </c>
-      <c r="G319" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/318.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -10084,7 +9692,7 @@
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>/data/legislator_images/319.jpg?v=7</t>
+          <t>/data/legislator_images/rep_sani_nazifi.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10112,11 +9720,7 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="G321" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/320.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -10142,11 +9746,7 @@
           <t>Jigawa</t>
         </is>
       </c>
-      <c r="G322" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/321.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -10174,7 +9774,7 @@
       </c>
       <c r="G323" t="inlineStr">
         <is>
-          <t>/data/legislator_images/322.jpg?v=7</t>
+          <t>/data/legislator_images/rep_amos_daniel.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10202,11 +9802,7 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="G324" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/323.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -10232,11 +9828,7 @@
           <t>Kaduna</t>
         </is>
       </c>
-      <c r="G325" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/324.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -10264,7 +9856,7 @@
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>/data/legislator_images/325.jpg?v=7</t>
+          <t>/data/legislator_images/rep_yahaya_suleiman_richifa.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10294,7 +9886,7 @@
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>/data/legislator_images/326.jpg?v=7</t>
+          <t>/data/legislator_images/rep_yusuf_badau.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10324,7 +9916,7 @@
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>/data/legislator_images/327.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abubakar_abubakar_kabir.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10352,11 +9944,7 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="G329" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/328.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -10382,11 +9970,7 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="G330" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/329.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -10412,11 +9996,7 @@
           <t>Kano</t>
         </is>
       </c>
-      <c r="G331" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/330.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -10442,11 +10022,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G332" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/331.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -10472,11 +10048,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G333" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/332.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -10502,11 +10074,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G334" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/333.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -10532,11 +10100,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G335" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/334.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -10564,7 +10128,7 @@
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>/data/legislator_images/335.jpg?v=7</t>
+          <t>/data/legislator_images/rep_murtala_usman_banye.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10592,11 +10156,7 @@
           <t>Katsina</t>
         </is>
       </c>
-      <c r="G337" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/336.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -10622,11 +10182,7 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="G338" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/337.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -10652,11 +10208,7 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="G339" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/338.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -10684,7 +10236,7 @@
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>/data/legislator_images/339.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ozigi_tijani.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10712,11 +10264,7 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="G341" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/340.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -10742,11 +10290,7 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="G342" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/341.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -10772,11 +10316,7 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="G343" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/342.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -10802,11 +10342,7 @@
           <t>Kebbi</t>
         </is>
       </c>
-      <c r="G344" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/343.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -10832,11 +10368,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G345" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/344.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -10864,7 +10396,7 @@
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>/data/legislator_images/345.jpg?v=7</t>
+          <t>/data/legislator_images/rep_thaddeus_attah.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10892,11 +10424,7 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="G347" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/346.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -10924,7 +10452,7 @@
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>/data/legislator_images/347.jpg?v=7</t>
+          <t>/data/legislator_images/rep_mohammed_bio.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -10952,11 +10480,7 @@
           <t>Kwara</t>
         </is>
       </c>
-      <c r="G349" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/348.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -10984,7 +10508,7 @@
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>/data/legislator_images/349.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ismail_kayode_tijani.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -11012,11 +10536,7 @@
           <t>Nasarawa</t>
         </is>
       </c>
-      <c r="G351" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/350.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -11044,7 +10564,7 @@
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>/data/legislator_images/351.jpg?v=7</t>
+          <t>/data/legislator_images/rep_abdullahi_idris_garba.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -11072,11 +10592,7 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="G353" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/352.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -11102,11 +10618,7 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="G354" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/353.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -11134,7 +10646,7 @@
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>/data/legislator_images/354.jpg?v=7</t>
+          <t>/data/legislator_images/rep_oladebo_lanre_olomololaye.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -11162,11 +10674,7 @@
           <t>Osun</t>
         </is>
       </c>
-      <c r="G356" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/355.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="n">
@@ -11192,11 +10700,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G357" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/356.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -11222,11 +10726,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G358" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/357.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="n">
@@ -11252,11 +10752,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G359" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/358.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="n">
@@ -11282,11 +10778,7 @@
           <t>Oyo</t>
         </is>
       </c>
-      <c r="G360" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/359.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -11312,11 +10804,7 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="G361" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/360.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="n">
@@ -11344,7 +10832,7 @@
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>/data/legislator_images/361.jpg?v=7</t>
+          <t>/data/legislator_images/rep_ajang_iliya.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -11372,11 +10860,7 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="G363" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/362.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -11402,11 +10886,7 @@
           <t>Rivers</t>
         </is>
       </c>
-      <c r="G364" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/363.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="n">
@@ -11432,11 +10912,7 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="G365" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/364.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -11464,7 +10940,7 @@
       </c>
       <c r="G366" t="inlineStr">
         <is>
-          <t>/data/legislator_images/365.jpg?v=7</t>
+          <t>/data/legislator_images/rep_nasiru_shehu_bodinga.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -11492,11 +10968,7 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="G367" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/366.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="n">
@@ -11527,11 +10999,7 @@
           <t>Cleaned &amp; Upscaled</t>
         </is>
       </c>
-      <c r="G368" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/367.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -11557,11 +11025,7 @@
           <t>Sokoto</t>
         </is>
       </c>
-      <c r="G369" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/368.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="n">
@@ -11587,11 +11051,7 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="G370" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/369.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="n">
@@ -11617,11 +11077,7 @@
           <t>Taraba</t>
         </is>
       </c>
-      <c r="G371" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/370.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="n">
@@ -11649,7 +11105,7 @@
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>/data/legislator_images/371.jpg?v=7</t>
+          <t>/data/legislator_images/rep_khadija_bukar_abba_ibrahim.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -11677,11 +11133,7 @@
           <t>Yobe</t>
         </is>
       </c>
-      <c r="G373" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/372.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="n">
@@ -11707,11 +11159,7 @@
           <t>Kogi</t>
         </is>
       </c>
-      <c r="G374" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/373.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="n">
@@ -11739,7 +11187,7 @@
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>/data/legislator_images/374.jpg?v=7</t>
+          <t>/data/legislator_images/rep_uchenna_clement_nwachukwu.jpg?v=11</t>
         </is>
       </c>
     </row>
@@ -11767,11 +11215,7 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="G376" t="inlineStr">
-        <is>
-          <t>/data/legislator_images/375.jpg?v=7</t>
-        </is>
-      </c>
+      <c r="G376" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>